<commit_message>
111.36.1: Excel-Ansicht – Bilder mit Zuschnitt und durchsichtiger Farbe wie in Excel
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Po9D778pv9LMBbksfwU1by
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-beispiel.xlsx
@@ -261,6 +261,62 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+        </a:blip>
+        <a:srcRect r="50000"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
111.44.0: Excel-Ansicht als A4-Seite mit Rändern, ganz eingepasst
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Po9D778pv9LMBbksfwU1by
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-beispiel.xlsx
@@ -8,6 +8,9 @@
     <sheet sheetId="2" name="Werkzeuge" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Versteckt" state="hidden" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Einrichtblatt'!$A1:$F16</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -642,6 +645,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -789,8 +795,8 @@
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="E2:F2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
111.52.0 Excel-Einrichtblätter wie in Excel: Textfelder und Formen, hoch-/tiefgestellt, Rahmenzeilen ohne Wert, Inhalt mittig mit gleichen Rändern
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014nGxBhHfr7VJVF1riHuxAq
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-beispiel.xlsx
@@ -150,7 +150,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -172,11 +172,18 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -197,6 +204,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -320,6 +328,64 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="900000" cy="220000"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="90" name="Textfeld 1"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="900000" cy="220000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:srgbClr val="C00000"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-CH" sz="1200" b="1"/>
+            <a:t>HD</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-CH" sz="1000"/>
+            <a:t> 4 mm</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-CH" sz="1000" baseline="30000"/>
+            <a:t>2</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -775,11 +841,19 @@
         <v>16</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+    </row>
     <row r="12" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="12">
         <f>SUM(E8:E10)</f>
         <v>4700</v>
       </c>
@@ -807,7 +881,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B1" t="s">
@@ -821,7 +895,7 @@
       <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="14">
         <v>0.25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
111.52.1 Excel-Ansicht: hoch- und tiefgestellte Zahlen kleiner und ganz sichtbar statt abgeschnitten
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014nGxBhHfr7VJVF1riHuxAq
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-beispiel.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Einrichtblatt 10844-0049</t>
   </si>
@@ -67,6 +67,31 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+      </rPr>
+      <t xml:space="preserve">6.80 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+      </rPr>
+      <t>+0.05</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+      </rPr>
+      <t xml:space="preserve"> -0.10</t>
+    </r>
   </si>
   <si>
     <t>Summe</t>
@@ -849,9 +874,12 @@
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
     </row>
-    <row r="12" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
       <c r="D12" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="12">
         <f>SUM(E8:E10)</f>
@@ -860,7 +888,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -882,18 +910,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="14">
         <v>0.25</v>
@@ -912,7 +940,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel-Ansicht: ausgeblendete Zeilen unsichtbar, An Zellgrösse anpassen (1.76.1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VwaR8f75EuToUQCeq5x6DF
</commit_message>
<xml_diff>
--- a/pruefstand/einrichtblatt-beispiel.xlsx
+++ b/pruefstand/einrichtblatt-beispiel.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Einrichtblatt 10844-0049</t>
   </si>
@@ -28,6 +28,9 @@
   </si>
   <si>
     <t>1.4305 V2A Ø 12 h9</t>
+  </si>
+  <si>
+    <t>DNMG 110408EN-M50 CTCP125-P</t>
   </si>
   <si>
     <t>Menge</t>
@@ -95,6 +98,9 @@
   </si>
   <si>
     <t>Summe</t>
+  </si>
+  <si>
+    <t>DNMU110404 MF1</t>
   </si>
   <si>
     <r>
@@ -208,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -218,6 +224,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -232,6 +241,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -770,125 +782,133 @@
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
+      <c r="D4" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5">
         <v>12500</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="F7" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+      <c r="A8" s="7">
         <v>1</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="7">
+      <c r="B8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="8">
         <v>3200</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="9">
         <v>0.08</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="8">
         <v>1500</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>12</v>
+      <c r="F8" s="10" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+      <c r="A9" s="7">
         <v>2</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="7">
+      <c r="B9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="8">
         <v>2800</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <v>0.035</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="8">
         <v>800</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>14</v>
+      <c r="F9" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+      <c r="A10" s="7">
         <v>3</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="7">
+      <c r="B10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="8">
         <v>4500</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>0.06</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="8">
         <v>2400</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>16</v>
+      <c r="F10" s="10" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="12">
+      <c r="D12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="13">
         <f>SUM(E8:E10)</f>
         <v>4700</v>
       </c>
     </row>
+    <row r="13" hidden="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="14" t="s">
+        <v>20</v>
+      </c>
+    </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -909,21 +929,21 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>20</v>
+      <c r="A1" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="14">
+        <v>25</v>
+      </c>
+      <c r="C2" s="16">
         <v>0.25</v>
       </c>
     </row>
@@ -940,7 +960,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>